<commit_message>
Hindalco: update PDFs & Excel (2026-09-17 08:47:44 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>368.75</v>
+        <v>373.25</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>12.09.2026</t>
+          <t>17.09.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-09-20 08:43:38 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>373.25</v>
+        <v>370.25</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>17.09.2026</t>
+          <t>19.09.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-september-2026.pdf</t>
         </is>
       </c>
     </row>
@@ -511,16 +511,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>373.25</v>
+        <v>370.25</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>17.09.2026</t>
+          <t>19.09.2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-september-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-09-22 08:41:33 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>370.25</v>
+        <v>367.75</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>19.09.2026</t>
+          <t>22.09.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-september-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-september-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-09-23 08:43:43 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>367.75</v>
+        <v>364.75</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>22.09.2026</t>
+          <t>23.09.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-september-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-09-30 05:50:24 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>366.25</v>
+        <v>363.75</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>26.09.2026</t>
+          <t>30.09.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-10-01 06:23:48 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>363.75</v>
+        <v>361.25</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>30.09.2026</t>
+          <t>01.10.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-october-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-10-02 06:01:18 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>361.25</v>
+        <v>352.5</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>01.10.2026</t>
+          <t>02.10.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-october-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-october-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-10-07 06:19:37 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>352.5</v>
+        <v>355.25</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>02.10.2026</t>
+          <t>07.10.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-october-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-october-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-10-08 06:31:04 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>355.25</v>
+        <v>352.5</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>07.10.2026</t>
+          <t>08.10.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-october-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-october-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-10-09 06:32:14 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>352.5</v>
+        <v>348.5</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>08.10.2026</t>
+          <t>09.10.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-october-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-10-13 07:00:03 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>348.5</v>
+        <v>344</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>09.10.2026</t>
+          <t>13.10.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-october-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-10-14 08:53:28 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>344</v>
+        <v>340.25</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>13.10.2026</t>
+          <t>14.10.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-october-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-october-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-10-15 08:28:14 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>340.25</v>
+        <v>336.5</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>14.10.2026</t>
+          <t>15.10.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-october-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-10-28 06:05:21 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>339.25</v>
+        <v>343.75</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>24.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-10-29 06:15:55 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>343.75</v>
+        <v>346.25</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>28.10.2026</t>
+          <t>29.10.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-october-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-10-30 06:16:49 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>346.25</v>
+        <v>343.75</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>29.10.2026</t>
+          <t>30.10.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-october-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>